<commit_message>
Add Certificaciones section and improve Quiénes somos on mobile/tablet
- New Certificaciones section (60 km): desktop replica of the design, flip
  cards (ISO 9001, ESR, Hecho en México), ES/EN texts, responsive layout
- Quiénes somos: more card padding, larger readable text on tablet/mobile,
  single-column help bar on mobile; desktop unchanged
- Docs, technical sheets and backlog updated

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LUTSA_Product_Backlog.xlsx
+++ b/docs/LUTSA_Product_Backlog.xlsx
@@ -853,7 +853,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rediseño web (landing + API) · Corte: 13/10/2026</t>
+          <t>Rediseño web (landing + API) · Corte: 16/10/2026</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="17" t="inlineStr">
         <is>
-          <t>2. Secciones de Galería y Certificaciones (requiere fotos y documentos de LUTSA).</t>
+          <t>2. Sección de Galería (requiere fotos de LUTSA y su diseño).</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Basado en «Requisitos para Rediseño Web» y en la revisión del código (landing + API LUTSA-CORE) · Corte: 13/10/2026 · Edita la columna «Avance %»: las barras y el resumen se actualizan solos</t>
+          <t>Basado en «Requisitos para Rediseño Web» y en la revisión del código (landing + API LUTSA-CORE) · Corte: 16/10/2026 · Edita la columna «Avance %»: las barras y el resumen se actualizan solos</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1937,7 @@
         <v>1</v>
       </c>
       <c r="G14" s="13" t="n">
-        <v>0.1</v>
+        <v>0.95</v>
       </c>
       <c r="H14" s="28">
         <f>REPT("█",ROUND(MAX(0,MIN(1,G14))*20,0))&amp;REPT("░",20-ROUND(MAX(0,MIN(1,G14))*20,0))</f>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="J14" s="27" t="inlineStr">
         <is>
-          <t>Solo existe el marcador. Falta diseño y logos/documentos de certificaciones.</t>
+          <t>Hecho: ISO 9001, ESR y Hecho en México con tarjetas que giran, igual al diseño y adaptado a móvil/tablet (ES/EN). Falta: validar textos oficiales con LUTSA.</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="J17" s="24" t="inlineStr">
         <is>
-          <t>Hecho: barra de km, Galería y Certificaciones (marcador). Falta: botón de WhatsApp y el contenido final de Galería/Certificaciones.</t>
+          <t>Hecho: barra de km, Certificaciones y Galería (marcador). Falta: botón de WhatsApp y el contenido final de Galería.</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="J33" s="24" t="inlineStr">
         <is>
-          <t>Ajustadas 6 de 8 secciones; faltan Galería y Certificaciones (aún son marcadores).</t>
+          <t>Ajustadas 7 de 8 secciones; falta Galería (aún es marcador).</t>
         </is>
       </c>
     </row>
@@ -3961,12 +3961,12 @@
       </c>
       <c r="C13" s="32" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Recibido</t>
         </is>
       </c>
       <c r="D13" s="31" t="inlineStr">
         <is>
-          <t>No viene en la lista del PDF, pero se necesita.</t>
+          <t>Logos ISO 9001, ESR y Hecho en México y foto de responsabilidad social. Falta confirmar textos oficiales.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reorder sections, mobile Servicios, subfolder deployment and UI tweaks
- Section order: Cotización at 50 km, Certificaciones 60 km, Galería 70 km
  (EN/ES titles and nav follow); Galería placeholder in its own component
- Cotización: captcha now below the submit button (desktop, tablet, mobile)
- Servicios on mobile: single centered column, larger text, full-width trailer cards
- Ecosistema on mobile/tablet: inactive circles get a navy veil instead of grayscale
- Support publishing in a subfolder: publicUrl() helper for public/ images,
  base path in routes/SEO/prerender, npm run build:pruebas -> dist-pruebas
  (noindex), root build unchanged
- Docs, backlog and style guide updated

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LUTSA_Product_Backlog.xlsx
+++ b/docs/LUTSA_Product_Backlog.xlsx
@@ -853,7 +853,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rediseño web (landing + API) · Corte: 16/10/2026</t>
+          <t>Rediseño web (landing + API) · Corte: 19/10/2026</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Basado en «Requisitos para Rediseño Web» y en la revisión del código (landing + API LUTSA-CORE) · Corte: 16/10/2026 · Edita la columna «Avance %»: las barras y el resumen se actualizan solos</t>
+          <t>Basado en «Requisitos para Rediseño Web» y en la revisión del código (landing + API LUTSA-CORE) · Corte: 19/10/2026 · Edita la columna «Avance %»: las barras y el resumen se actualizan solos</t>
         </is>
       </c>
     </row>
@@ -1903,7 +1903,7 @@
       </c>
       <c r="J13" s="24" t="inlineStr">
         <is>
-          <t>Solo existe el marcador y su parada en la barra de km. Falta diseño y fotos (requiere material de LUTSA). Va antes de Certificaciones.</t>
+          <t>Solo existe el marcador y su parada en la barra de km. Falta diseño y fotos (requiere material de LUTSA). Ahora es la última sección (70 km); la Cotización pasó al 50 km.</t>
         </is>
       </c>
     </row>

</xml_diff>